<commit_message>
v0.1.1: class definitions, facet-property inverses/domains, upper-class disjointness; add reasoner, OOPS!, parser-validation and trend-statistics scripts and outputs
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/design/OSA_ontology_class_design.xlsx
+++ b/design/OSA_ontology_class_design.xlsx
@@ -10444,7 +10444,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R118" t="inlineStr">
@@ -60010,7 +60010,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -60235,7 +60235,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -60460,7 +60460,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -60685,7 +60685,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -63512,7 +63512,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -63737,7 +63737,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -63962,7 +63962,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -64187,7 +64187,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>각성무관</t>
+          <t>각성포함</t>
         </is>
       </c>
       <c r="R74" t="inlineStr">
@@ -64257,7 +64257,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -64332,7 +64332,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -64407,7 +64407,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -64482,7 +64482,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -65536,7 +65536,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -65611,7 +65611,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -65686,7 +65686,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -65761,7 +65761,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -65986,7 +65986,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -66061,7 +66061,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
@@ -66136,7 +66136,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -66211,7 +66211,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>전체/무기준</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">

</xml_diff>